<commit_message>
Daily NSE scan: 2026-10-06
</commit_message>
<xml_diff>
--- a/output/2026-10-06/enriched_analysis.xlsx
+++ b/output/2026-10-06/enriched_analysis.xlsx
@@ -1161,10 +1161,10 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>2.2</v>
+        <v>2.201</v>
       </c>
       <c r="W3" t="n">
-        <v>2864</v>
+        <v>2863</v>
       </c>
       <c r="X3" t="n">
         <v>22.4</v>
@@ -1393,13 +1393,13 @@
         </is>
       </c>
       <c r="V4" t="n">
-        <v>1.155</v>
+        <v>1.159</v>
       </c>
       <c r="W4" t="n">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="X4" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="Y4" t="n">
         <v>22</v>
@@ -2093,7 +2093,7 @@
         <v>922</v>
       </c>
       <c r="X7" t="n">
-        <v>9.06</v>
+        <v>9.07</v>
       </c>
       <c r="Y7" t="n">
         <v>7</v>
@@ -2319,10 +2319,10 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.533</v>
+        <v>0.532</v>
       </c>
       <c r="W8" t="n">
-        <v>2681</v>
+        <v>2682</v>
       </c>
       <c r="X8" t="n">
         <v>22</v>
@@ -2551,13 +2551,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>1.091</v>
+        <v>1.062</v>
       </c>
       <c r="W9" t="n">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="X9" t="n">
-        <v>7.83</v>
+        <v>8.01</v>
       </c>
       <c r="Y9" t="n">
         <v>17</v>
@@ -2786,10 +2786,10 @@
         <v>0.049</v>
       </c>
       <c r="W10" t="n">
-        <v>14738</v>
+        <v>14755</v>
       </c>
       <c r="X10" t="n">
-        <v>37.5</v>
+        <v>37.6</v>
       </c>
       <c r="Y10" t="n">
         <v>83</v>
@@ -3018,7 +3018,7 @@
         <v>0.128</v>
       </c>
       <c r="W11" t="n">
-        <v>2447</v>
+        <v>2446</v>
       </c>
       <c r="X11" t="n">
         <v>21.4</v>
@@ -3247,13 +3247,13 @@
         </is>
       </c>
       <c r="V12" t="n">
-        <v>2.305</v>
+        <v>2.316</v>
       </c>
       <c r="W12" t="n">
-        <v>2547</v>
+        <v>2534</v>
       </c>
       <c r="X12" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Y12" t="n">
         <v>6</v>
@@ -3479,13 +3479,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>2.783</v>
+        <v>2.787</v>
       </c>
       <c r="W13" t="n">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="X13" t="n">
-        <v>26.6</v>
+        <v>26.5</v>
       </c>
       <c r="Y13" t="n">
         <v>30</v>
@@ -3705,13 +3705,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.067</v>
+        <v>0.066</v>
       </c>
       <c r="W14" t="n">
-        <v>838</v>
+        <v>858</v>
       </c>
       <c r="X14" t="n">
-        <v>21.2</v>
+        <v>21.7</v>
       </c>
       <c r="Y14" t="n">
         <v>19</v>
@@ -3938,7 +3938,7 @@
         <v>0.052</v>
       </c>
       <c r="W15" t="n">
-        <v>1588</v>
+        <v>1591</v>
       </c>
       <c r="X15" t="n">
         <v>21.4</v>
@@ -4170,10 +4170,10 @@
         <v>0.064</v>
       </c>
       <c r="W16" t="n">
-        <v>1732</v>
+        <v>1742</v>
       </c>
       <c r="X16" t="n">
-        <v>39.8</v>
+        <v>40</v>
       </c>
       <c r="Y16" t="n">
         <v>20</v>
@@ -4402,10 +4402,10 @@
         <v>0.129</v>
       </c>
       <c r="W17" t="n">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="X17" t="n">
-        <v>29</v>
+        <v>29.1</v>
       </c>
       <c r="Y17" t="n">
         <v>17</v>
@@ -4628,7 +4628,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W18" t="n">
-        <v>53461</v>
+        <v>53450</v>
       </c>
       <c r="X18" t="n">
         <v>45.3</v>
@@ -4857,13 +4857,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.199</v>
+        <v>0.192</v>
       </c>
       <c r="W19" t="n">
-        <v>556</v>
+        <v>578</v>
       </c>
       <c r="X19" t="n">
-        <v>46.5</v>
+        <v>48.3</v>
       </c>
       <c r="Y19" t="n">
         <v>3</v>
@@ -5089,10 +5089,10 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.089</v>
+        <v>0.09</v>
       </c>
       <c r="W20" t="n">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="X20" t="n">
         <v>10.4</v>
@@ -5324,7 +5324,7 @@
         <v>0.375</v>
       </c>
       <c r="W21" t="n">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="X21" t="n">
         <v>53.4</v>
@@ -5553,10 +5553,10 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.67</v>
+        <v>0.668</v>
       </c>
       <c r="W22" t="n">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="X22" t="n">
         <v>10.8</v>
@@ -5785,13 +5785,13 @@
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.517</v>
+        <v>0.513</v>
       </c>
       <c r="W23" t="n">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="X23" t="n">
-        <v>35.8</v>
+        <v>36.1</v>
       </c>
       <c r="Y23" t="n">
         <v>21</v>
@@ -6017,13 +6017,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.332</v>
+        <v>0.334</v>
       </c>
       <c r="W24" t="n">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="X24" t="n">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="Y24" t="n">
         <v>12</v>
@@ -6249,13 +6249,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.287</v>
+        <v>0.286</v>
       </c>
       <c r="W25" t="n">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="X25" t="n">
-        <v>24.7</v>
+        <v>24.8</v>
       </c>
       <c r="Y25" t="n">
         <v>9</v>
@@ -6481,13 +6481,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.982</v>
+        <v>0.977</v>
       </c>
       <c r="W26" t="n">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="X26" t="n">
-        <v>5.91</v>
+        <v>5.93</v>
       </c>
       <c r="Y26" t="n">
         <v>31</v>
@@ -7171,10 +7171,10 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.135</v>
+        <v>0.134</v>
       </c>
       <c r="W29" t="n">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="X29" t="n">
         <v>13.1</v>
@@ -7406,10 +7406,10 @@
         <v>0.044</v>
       </c>
       <c r="W30" t="n">
-        <v>1591</v>
+        <v>1586</v>
       </c>
       <c r="X30" t="n">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="Y30" t="n">
         <v>10</v>
@@ -7867,13 +7867,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.234</v>
+        <v>0.233</v>
       </c>
       <c r="W32" t="n">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="X32" t="n">
-        <v>14.6</v>
+        <v>14.7</v>
       </c>
       <c r="Y32" t="n">
         <v>16</v>
@@ -8099,13 +8099,13 @@
         </is>
       </c>
       <c r="V33" t="n">
-        <v>0.677</v>
+        <v>0.667</v>
       </c>
       <c r="W33" t="n">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="X33" t="n">
-        <v>1120</v>
+        <v>1137</v>
       </c>
       <c r="Y33" t="n">
         <v>-61</v>
@@ -8327,13 +8327,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.373</v>
+        <v>0.374</v>
       </c>
       <c r="W34" t="n">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="X34" t="n">
-        <v>92.7</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="Y34" t="n">
         <v>246</v>
@@ -8788,10 +8788,10 @@
         <v>0.233</v>
       </c>
       <c r="W36" t="n">
-        <v>1716</v>
+        <v>1715</v>
       </c>
       <c r="X36" t="n">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="Y36" t="n">
         <v>-3</v>
@@ -9020,7 +9020,7 @@
         <v>0.042</v>
       </c>
       <c r="W37" t="n">
-        <v>3168</v>
+        <v>3170</v>
       </c>
       <c r="X37" t="n">
         <v>18.8</v>
@@ -9252,7 +9252,7 @@
         <v>0.011</v>
       </c>
       <c r="W38" t="n">
-        <v>4209</v>
+        <v>4185</v>
       </c>
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="n">
@@ -9482,7 +9482,7 @@
         <v>0</v>
       </c>
       <c r="W39" t="n">
-        <v>4988</v>
+        <v>4986</v>
       </c>
       <c r="X39" t="n">
         <v>11.7</v>
@@ -9714,10 +9714,10 @@
         <v>0.109</v>
       </c>
       <c r="W40" t="n">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="X40" t="n">
-        <v>7.33</v>
+        <v>7.37</v>
       </c>
       <c r="Y40" t="n">
         <v>118</v>
@@ -9942,10 +9942,10 @@
         <v>0.078</v>
       </c>
       <c r="W41" t="n">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="X41" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="Y41" t="n">
         <v>-8</v>
@@ -10403,10 +10403,10 @@
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.052</v>
+        <v>0.053</v>
       </c>
       <c r="W43" t="n">
-        <v>943</v>
+        <v>937</v>
       </c>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="n">
@@ -10868,7 +10868,7 @@
         <v>0.006</v>
       </c>
       <c r="W45" t="n">
-        <v>4853</v>
+        <v>4858</v>
       </c>
       <c r="X45" t="n">
         <v>12.5</v>
@@ -11096,10 +11096,10 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>3844</v>
+        <v>3825</v>
       </c>
       <c r="X46" t="n">
-        <v>86.5</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="Y46" t="n">
         <v>42</v>
@@ -11325,13 +11325,13 @@
         </is>
       </c>
       <c r="V47" t="n">
-        <v>0.218</v>
+        <v>0.217</v>
       </c>
       <c r="W47" t="n">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="X47" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="Y47" t="n">
         <v>21</v>
@@ -11560,10 +11560,10 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>112087</v>
+        <v>111934</v>
       </c>
       <c r="X48" t="n">
-        <v>32.3</v>
+        <v>32.2</v>
       </c>
       <c r="Y48" t="n">
         <v>18</v>

</xml_diff>